<commit_message>
Preserve partial import on stop, warn on missing SSD thresholds, update soglie
- On user stop: keep run directory and collected JSONs instead of deleting;
  write metadata.json with aborted:true; dropdown shows ⚠️ label for aborted runs
- Remove now-unused _cleanup_run_directory and shutil import
- Log warning when member SSD has no entry in soglie.xlsx
- Update soglie.xlsx with correct data for all 11 SSDs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/soglie/soglie.xlsx
+++ b/soglie/soglie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/riccardoberta/Source/Diten/DEEP/soglie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350E61B3-8D30-EE47-B989-1BBAC9A800F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0E54DF-6498-DC45-B957-62B17FDA1356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1880" yWindow="4300" windowWidth="30240" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Soglie" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="76">
   <si>
     <t>ELETTROTECNICA</t>
   </si>
@@ -212,6 +212,42 @@
   </si>
   <si>
     <t>H-idx 15a - I</t>
+  </si>
+  <si>
+    <t>06/MEDS-16</t>
+  </si>
+  <si>
+    <t>MALATTIE ODONTOSTOMATOLOGICHE</t>
+  </si>
+  <si>
+    <t>MEDS-16/A</t>
+  </si>
+  <si>
+    <t>Malattie odontostomatologiche</t>
+  </si>
+  <si>
+    <t>06/F1 - MALATTIE ODONTOSTOMATOLOGICHE</t>
+  </si>
+  <si>
+    <t>MED/28 - MALATTIE ODONTOSTOMATOLOGICHE</t>
+  </si>
+  <si>
+    <t>01/INFO-01</t>
+  </si>
+  <si>
+    <t>INFORMATICA</t>
+  </si>
+  <si>
+    <t>INFO-01/A</t>
+  </si>
+  <si>
+    <t>Informatica</t>
+  </si>
+  <si>
+    <t>01/B1 INFORMATICA</t>
+  </si>
+  <si>
+    <t>INF/01 - INFORMATICA</t>
   </si>
 </sst>
 </file>
@@ -240,7 +276,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -263,13 +299,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -575,7 +623,7 @@
   <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="44.5" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="48.5" customWidth="1"/>
@@ -1061,6 +1109,100 @@
         <v>13</v>
       </c>
     </row>
+    <row r="11" spans="1:15" ht="17">
+      <c r="A11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="1">
+        <v>14</v>
+      </c>
+      <c r="H11" s="1">
+        <v>143</v>
+      </c>
+      <c r="I11" s="1">
+        <v>6</v>
+      </c>
+      <c r="J11" s="1">
+        <v>20</v>
+      </c>
+      <c r="K11" s="1">
+        <v>202</v>
+      </c>
+      <c r="L11" s="1">
+        <v>8</v>
+      </c>
+      <c r="M11" s="1">
+        <v>28</v>
+      </c>
+      <c r="N11" s="1">
+        <v>482</v>
+      </c>
+      <c r="O11" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="17">
+      <c r="A12" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="1">
+        <v>4</v>
+      </c>
+      <c r="H12" s="1">
+        <v>157</v>
+      </c>
+      <c r="I12" s="1">
+        <v>7</v>
+      </c>
+      <c r="J12" s="1">
+        <v>9</v>
+      </c>
+      <c r="K12" s="1">
+        <v>304</v>
+      </c>
+      <c r="L12" s="1">
+        <v>10</v>
+      </c>
+      <c r="M12" s="1">
+        <v>11</v>
+      </c>
+      <c r="N12" s="1">
+        <v>391</v>
+      </c>
+      <c r="O12" s="1">
+        <v>11</v>
+      </c>
+    </row>
     <row r="21" spans="6:6">
       <c r="F21" t="s">
         <v>54</v>

</xml_diff>